<commit_message>
Add admin paging and secure admin config
</commit_message>
<xml_diff>
--- a/templates/google-sheet-template.xlsx
+++ b/templates/google-sheet-template.xlsx
@@ -1433,7 +1433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1442,7 +1442,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Huong dan cap nhat du lieu v4</t>
+          <t>Huong dan cap nhat du lieu v5 admin</t>
         </is>
       </c>
     </row>
@@ -1477,35 +1477,56 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5. App chi cong nhan dat muc khi ca 4 loai thue bao cua muc do deu dat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Tai khoan test:</t>
+          <t>5. Tai khoan admin duoc cau hinh trong file .env cua app, khong luu trong Google Sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>6. App chi cong nhan dat muc khi ca 4 loai thue bao cua muc do deu dat.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CUSPS0001 / 123456</t>
+          <t>Tai khoan test diem ban:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CUSPS0002 / abc789</t>
+          <t>CUSPS0001 / 123456</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>CUSPS0002 / abc789</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>CUSPS0003 / pdv2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tai khoan admin mau trong .env.example:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ADMIN01 / change-this-admin-password</t>
         </is>
       </c>
     </row>

</xml_diff>